<commit_message>
MAJ pipeline 2026-07-28 14:04
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-28.xlsx
+++ b/jira_export_2026-07-28.xlsx
@@ -732,7 +732,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>58,312 €</t>
+          <t>60,001 €</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -746,7 +746,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>63.2%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -772,7 +772,7 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>20,214 €</t>
+          <t>21,902 €</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
@@ -827,7 +827,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>537 h</t>
+          <t>539 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -841,7 +841,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>70.7%</t>
+          <t>71.0%</t>
         </is>
       </c>
       <c r="H16" s="7" t="n"/>
@@ -1633,10 +1633,10 @@
         <v>430</v>
       </c>
       <c r="O12" s="16" t="n">
-        <v>860</v>
+        <v>1978</v>
       </c>
       <c r="P12" s="16" t="n">
-        <v>70.2</v>
+        <v>161.47</v>
       </c>
     </row>
     <row r="13">
@@ -3185,10 +3185,10 @@
         <v>1242.9</v>
       </c>
       <c r="O34" s="17" t="n">
-        <v>621.45</v>
+        <v>870.03</v>
       </c>
       <c r="P34" s="16" t="n">
-        <v>62.15</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35">
@@ -3833,10 +3833,10 @@
         <v>920</v>
       </c>
       <c r="O43" s="17" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
       <c r="P43" s="13" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44">
@@ -5033,7 +5033,7 @@
         <v>2</v>
       </c>
       <c r="K60" s="15" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="L60" s="15" t="inlineStr">
         <is>
@@ -5105,7 +5105,7 @@
         <v>2</v>
       </c>
       <c r="K61" s="12" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="L61" s="12" t="inlineStr">
         <is>
@@ -5124,7 +5124,7 @@
         <v>224</v>
       </c>
       <c r="P61" s="13" t="n">
-        <v>896</v>
+        <v>298.67</v>
       </c>
     </row>
     <row r="62">
@@ -11357,7 +11357,7 @@
         <v>15</v>
       </c>
       <c r="K149" s="12" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="L149" s="12" t="inlineStr">
         <is>
@@ -13691,10 +13691,10 @@
         <v>65939.26000000001</v>
       </c>
       <c r="O186" s="19" t="n">
-        <v>58312.215</v>
+        <v>60000.79500000001</v>
       </c>
       <c r="P186" s="19" t="n">
-        <v>175.24</v>
+        <v>178.97</v>
       </c>
     </row>
   </sheetData>
@@ -14908,7 +14908,7 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>184.75</v>
+        <v>187.25</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>33.75</v>
@@ -14917,7 +14917,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>221.5</v>
+        <v>224</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>65.5</v>
@@ -14927,7 +14927,7 @@
       </c>
       <c r="H5" s="22" t="inlineStr">
         <is>
-          <t>45.6%</t>
+          <t>46.1%</t>
         </is>
       </c>
     </row>
@@ -15054,10 +15054,10 @@
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>382463</v>
+        <v>381275</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>125316</v>
+        <v>124127</v>
       </c>
       <c r="D5" s="25" t="n">
         <v>257148</v>
@@ -15079,10 +15079,10 @@
         </is>
       </c>
       <c r="B6" s="26" t="n">
-        <v>175491</v>
+        <v>174303</v>
       </c>
       <c r="C6" s="26" t="n">
-        <v>69609</v>
+        <v>68421</v>
       </c>
       <c r="D6" s="26" t="n">
         <v>105882</v>
@@ -15133,7 +15133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15157,7 +15157,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Épics créées ce mois — 17 commande(s)</t>
+          <t>Épics créées ce mois — 18 commande(s)</t>
         </is>
       </c>
     </row>
@@ -15212,22 +15212,22 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34768</t>
+          <t>PDMDEP-34621</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34761</t>
+          <t>PDMDEP-34613</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>20/07/2026</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DU PUY EN VELAY</t>
+          <t>COMMUNE DE FORT-DE-FRANCE</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -15237,7 +15237,7 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -15247,11 +15247,11 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>00177029</t>
+          <t>00176431</t>
         </is>
       </c>
       <c r="I5" s="26" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="6">
@@ -15482,22 +15482,22 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34420</t>
+          <t>PDMDEP-34589</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34411</t>
+          <t>PDMDEP-34580</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>16/07/2026</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>MAIRIE DE MAIZIERES LES METZ</t>
+          <t>COMMUNE DE RIEZ</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -15517,32 +15517,32 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>00172317</t>
+          <t>00176128</t>
         </is>
       </c>
       <c r="I11" s="26" t="n">
-        <v>2035</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34589</t>
+          <t>PDMDEP-34420</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34580</t>
+          <t>PDMDEP-34411</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>16/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>COMMUNE DE RIEZ</t>
+          <t>MAIRIE DE MAIZIERES LES METZ</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -15562,32 +15562,32 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>00176128</t>
+          <t>00172317</t>
         </is>
       </c>
       <c r="I12" s="27" t="n">
-        <v>1300</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34640</t>
+          <t>PDMDEP-34396</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34631</t>
+          <t>PDMDEP-34390</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
+          <t>Commune Le THOR</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -15607,11 +15607,11 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>00176477</t>
+          <t>00171793</t>
         </is>
       </c>
       <c r="I13" s="26" t="n">
-        <v>2250</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14">
@@ -15752,22 +15752,22 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34621</t>
+          <t>PDMDEP-34768</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34613</t>
+          <t>PDMDEP-34761</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>20/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DE FORT-DE-FRANCE</t>
+          <t>COMMUNE DU PUY EN VELAY</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -15777,7 +15777,7 @@
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -15787,32 +15787,32 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>00176431</t>
+          <t>00177029</t>
         </is>
       </c>
       <c r="I17" s="26" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34396</t>
+          <t>PDMDEP-34640</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34390</t>
+          <t>PDMDEP-34631</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Commune Le THOR</t>
+          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -15822,7 +15822,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -15832,11 +15832,11 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>00171793</t>
+          <t>00176477</t>
         </is>
       </c>
       <c r="I18" s="27" t="n">
-        <v>250</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="19">
@@ -15975,30 +15975,42 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>17 commande(s)</t>
-        </is>
-      </c>
-      <c r="I22" s="25" t="n">
-        <v>35552</v>
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>PDMDEP-34778</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>PSC-1315</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Rang-du-Fliers</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr"/>
+      <c r="G22" s="12" t="inlineStr"/>
+      <c r="H22" s="12" t="inlineStr"/>
+      <c r="I22" s="27" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>dont Littéralis</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B23" s="18" t="n"/>
@@ -16009,17 +16021,17 @@
       <c r="G23" s="18" t="n"/>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>3 commande(s)</t>
+          <t>18 commande(s)</t>
         </is>
       </c>
       <c r="I23" s="25" t="n">
-        <v>7595</v>
+        <v>36052</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>dont GEODP</t>
+          <t>dont Littéralis</t>
         </is>
       </c>
       <c r="B24" s="18" t="n"/>
@@ -16030,10 +16042,31 @@
       <c r="G24" s="18" t="n"/>
       <c r="H24" s="18" t="inlineStr">
         <is>
+          <t>4 commande(s)</t>
+        </is>
+      </c>
+      <c r="I24" s="25" t="n">
+        <v>8095</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>dont GEODP</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n"/>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
           <t>14 commande(s)</t>
         </is>
       </c>
-      <c r="I24" s="25" t="n">
+      <c r="I25" s="25" t="n">
         <v>27958</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MAJ pipeline 2026-07-28 22:04
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-28.xlsx
+++ b/jira_export_2026-07-28.xlsx
@@ -732,7 +732,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>60,001 €</t>
+          <t>60,145 €</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -746,7 +746,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>63.2%</t>
+          <t>63.3%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -772,7 +772,7 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>21,902 €</t>
+          <t>22,046 €</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
@@ -827,7 +827,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>539 h</t>
+          <t>547 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -841,7 +841,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>72.1%</t>
         </is>
       </c>
       <c r="H16" s="7" t="n"/>
@@ -2337,10 +2337,10 @@
         <v>1296</v>
       </c>
       <c r="O22" s="16" t="n">
-        <v>2232</v>
+        <v>2376</v>
       </c>
       <c r="P22" s="16" t="n">
-        <v>156.63</v>
+        <v>166.74</v>
       </c>
     </row>
     <row r="23">
@@ -8405,7 +8405,7 @@
         <v>6</v>
       </c>
       <c r="K107" s="12" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="L107" s="12" t="inlineStr">
         <is>
@@ -9193,7 +9193,7 @@
         <v>8</v>
       </c>
       <c r="K118" s="15" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="L118" s="15" t="inlineStr">
         <is>
@@ -9212,7 +9212,7 @@
         <v>3453.22</v>
       </c>
       <c r="P118" s="16" t="n">
-        <v>1151.07</v>
+        <v>986.63</v>
       </c>
     </row>
     <row r="119">
@@ -9265,7 +9265,7 @@
         <v>8</v>
       </c>
       <c r="K119" s="12" t="n">
-        <v>1.15</v>
+        <v>1.25</v>
       </c>
       <c r="L119" s="12" t="inlineStr">
         <is>
@@ -9337,7 +9337,7 @@
         <v>8</v>
       </c>
       <c r="K120" s="15" t="n">
-        <v>1.15</v>
+        <v>1.25</v>
       </c>
       <c r="L120" s="15" t="inlineStr">
         <is>
@@ -9409,7 +9409,7 @@
         <v>8</v>
       </c>
       <c r="K121" s="12" t="n">
-        <v>1.15</v>
+        <v>1.25</v>
       </c>
       <c r="L121" s="12" t="inlineStr">
         <is>
@@ -9481,7 +9481,7 @@
         <v>8</v>
       </c>
       <c r="K122" s="15" t="n">
-        <v>1.15</v>
+        <v>1.25</v>
       </c>
       <c r="L122" s="15" t="inlineStr">
         <is>
@@ -9553,7 +9553,7 @@
         <v>8</v>
       </c>
       <c r="K123" s="12" t="n">
-        <v>1.15</v>
+        <v>1.25</v>
       </c>
       <c r="L123" s="12" t="inlineStr">
         <is>
@@ -9623,7 +9623,7 @@
         <v>8</v>
       </c>
       <c r="K124" s="15" t="n">
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="L124" s="15" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
         <v>29</v>
       </c>
       <c r="K169" s="12" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="L169" s="12" t="inlineStr"/>
       <c r="M169" s="12" t="inlineStr"/>
@@ -12821,7 +12821,7 @@
         <v>30</v>
       </c>
       <c r="K171" s="12" t="n">
-        <v>7.25</v>
+        <v>7.75</v>
       </c>
       <c r="L171" s="12" t="inlineStr"/>
       <c r="M171" s="12" t="inlineStr"/>
@@ -13691,10 +13691,10 @@
         <v>65939.26000000001</v>
       </c>
       <c r="O186" s="19" t="n">
-        <v>60000.79500000001</v>
+        <v>60144.79500000001</v>
       </c>
       <c r="P186" s="19" t="n">
-        <v>178.97</v>
+        <v>177.94</v>
       </c>
     </row>
   </sheetData>
@@ -14908,16 +14908,16 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>187.25</v>
+        <v>189</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>33.75</v>
+        <v>34.75</v>
       </c>
       <c r="D5" s="15" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>224</v>
+        <v>226.75</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>65.5</v>
@@ -14927,7 +14927,7 @@
       </c>
       <c r="H5" s="22" t="inlineStr">
         <is>
-          <t>46.1%</t>
+          <t>46.6%</t>
         </is>
       </c>
     </row>
@@ -14969,7 +14969,7 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>114.58</v>
+        <v>119.83</v>
       </c>
     </row>
   </sheetData>
@@ -15054,16 +15054,16 @@
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>381275</v>
+        <v>381131</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>124127</v>
+        <v>122302</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>257148</v>
+        <v>258828</v>
       </c>
       <c r="E5" s="25" t="n">
-        <v>165176</v>
+        <v>166857</v>
       </c>
       <c r="F5" s="25" t="n">
         <v>22749</v>
@@ -15079,10 +15079,10 @@
         </is>
       </c>
       <c r="B6" s="26" t="n">
-        <v>174303</v>
+        <v>174159</v>
       </c>
       <c r="C6" s="26" t="n">
-        <v>68421</v>
+        <v>68277</v>
       </c>
       <c r="D6" s="26" t="n">
         <v>105882</v>
@@ -15107,13 +15107,13 @@
         <v>206972</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>55706</v>
+        <v>54026</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>151265</v>
+        <v>152946</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>77690</v>
+        <v>79371</v>
       </c>
       <c r="F7" s="27" t="n">
         <v>10557</v>

</xml_diff>